<commit_message>
Add a full item-by-item walkthrough for one entity
Every finding against Motilal Oswal with its obligation source, method,
evidence, what it supports and what it explicitly does not -- the form needed if
the entity's compliance officer or counsel asks.

Two findings would survive challenge: no accessibility-specific grievance
mechanism, and three untagged Investor Charter PDFs. Both rest on provisions in
force since 31 July 2025 that the October extension did not move. The absence of
an accessibility statement is recorded as a transparency observation only, since
SEBI requires none.

Records a failure caught mid-walkthrough: a re-verification without --compressed
analysed gzip bytes and appeared to show the PDFs were unreadable scanned images.
That would have been false. Text is extractable from all three.
</commit_message>
<xml_diff>
--- a/evidence/claim-verification.xlsx
+++ b/evidence/claim-verification.xlsx
@@ -1,23 +1,39 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
-  <fileVersion appName="Calc" lowestEdited="4"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sanjayc/sebi-regulated-entity-accessibility/evidence/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AC97CCF-1885-AB44-B0B2-1D7F7EB3626F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17300" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Claims" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Broker Data" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="Charters" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="Circulars" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Claims" sheetId="1" r:id="rId1"/>
+    <sheet name="Broker Data" sheetId="2" r:id="rId2"/>
+    <sheet name="Charters" sheetId="3" r:id="rId3"/>
+    <sheet name="Circulars" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Claims!$A$1:$I$49</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Claims!$A$1:$I$49</definedName>
   </definedNames>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
     </ext>
@@ -28,1022 +44,1019 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="626" uniqueCount="336">
   <si>
-    <t xml:space="preserve">ID</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Claim</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Where it appears</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Category</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Status</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Evidence</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Source</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Verified</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Correction / note</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Supreme Court, 30 Apr 2025, held the right to digital access an intrinsic component of the right to life and personal liberty</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Article; guide Ch.3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Regulation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VERIFIED</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Quoted verbatim inside the circular itself</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SEBI 2025/111 Annexure I s.A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-08-20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The case is Pragya Prasun &amp; Ors. v. Union of India, heard with a Jain matter</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Article; guide</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NARROWER</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Circular names 'Pragya Prasun &amp; Ors.' and 'Jain vs. Union of India'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">First name 'Amar' comes from secondary coverage only. Article corrected to 'a Jain matter'.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Standards are WCAG 2.1 or latest, GIGW latest, IS 17802, RPwD Act</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Article; guide Ch.4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Verbatim, four numbered items</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SEBI 2025/111 Annexure I s.B</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SEBI never writes WCAG 2.2, GIGW 3.0, or a year for IS 17802</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Article</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Full text of four circulars searched</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025/111, 2025/121, 2025/131, Dec 2025</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A Nodal Officer for digital accessibility is mandatory</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Verbatim</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025/111 s.1.1-1.2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">An accessibility-specific grievance mechanism with escalation is required</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025/111 s.1.3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Investor PDFs must follow accessible document standards; circular cites the WCAG PDF techniques</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Verbatim, with the W3C URL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025/111 s.2.2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ISL, captions, descriptive audio and alt text are required</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025/111 s.2.1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Audits must include usability testing by persons with disabilities</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025/111 s.5.1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A disabled applicant may be rejected only after human review, with power to override automation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025/111 s.4.2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Responsibility for platform accessibility stays with the RE even for SaaS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The circular says 'responsibility', not 'liability'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025/111 s.6.1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Article corrected: 'liability' replaced in two places.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Audit and remediation deadline is 31 October 2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Circular reproduced inside an exchange notice</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HO/(411)2026-ITD-5_DIV2/I/17922/2026 via BSE Notice 20260731-17</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The 14 Dec 2025 auditor milestone was replaced, not supplemented</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Verbatim: 'Instead of meeting the compliance requirement...'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dec 2025 clarification para 3(a)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Compliance is filed by email to SEBI, an exchange or a depository</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Article; guide Ch.5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Submission mechanism and formats prescribed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025/131 Part B; Dec 2025 Annexure A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The circulars prescribe no penalty</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Issued under s.11(1); no penalty clause in any circular read</t>
-  </si>
-  <si>
-    <t xml:space="preserve">All five read</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vendor claims of a penalty regime describe SEBI's general powers.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">'Six circulars'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Article v1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CORRECTED</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SEBI's own Dec clarification references three prior circulars; the May 2025 KYC circular is a different series (MIRSD)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dec 2025 clarification reference table</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Corrected to: five digital accessibility circulars, preceded by a KYC circular.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R17</t>
-  </si>
-  <si>
-    <t xml:space="preserve">'Nothing in six circulars requires publication'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">One of the six has not been read against primary text</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OQ-3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Narrowed to the five actually read.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">24 obligations: 7 public, 4 artifact, 2 client, 11 not observable</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Article; repo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Classification</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Own classification, published in full</t>
-  </si>
-  <si>
-    <t xml:space="preserve">regulation/obligations.md</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Presented as a classification, not a finding of fact. 7+4+2+11=24.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SEBI's own Investor Charter contains no digital accessibility right</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Charter</t>
-  </si>
-  <si>
-    <t xml:space="preserve">64,777 chars retrieved; zero matches for 'digital accessib' or 'disabilit'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">investor.sebi.gov.in/Investor-charter.html</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The most recent Investor Charter circular for stock brokers is 21 Feb 2025</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Circular located; Dec 2025 to May 2026 window not exhaustively searched</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SEBI/HO/MIRSD/MIRSD-PoD1/P/CIR/2025/22</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keep the hedge 'that I can locate'. Tracked as OQ-1.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">'Eleven brokers' charters'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ten. 5paisa returns HTTP 403 and no charter was retrievable</t>
-  </si>
-  <si>
-    <t xml:space="preserve">out/charter-verification.json</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Corrected throughout the article.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">None of the charters checked contains the digital accessibility right</t>
-  </si>
-  <si>
-    <t xml:space="preserve">32 documents, 10 brokers, ~414,000 chars, whitespace-normalised. Zero matches</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">'Every charter is the standard SEBI template, word for word'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Only 7 of 10 carry the legacy clause XVII</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Removed; replaced with the claim actually evidenced.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Corpus adequacy for two brokers</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kotak 2,728 chars and HDFC 5,874 are thin; likely landing pages not full charters</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Stated as a caveat in the article.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">In Angel One's charter neither 'accessib' nor 'disab' appears</t>
-  </si>
-  <si>
-    <t xml:space="preserve">34,416 chars, neither string present</t>
-  </si>
-  <si>
-    <t xml:space="preserve">out/charters/angel-one.txt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Of the brokers checked, one publishes an accessibility statement</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Article; guide Ch.6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Disclosure</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kotak Securities; page retrieved and read in full</t>
-  </si>
-  <si>
-    <t xml:space="preserve">kotakneo.com/disclaimer/web-accessibility-statement/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kotak's statement names Pivotal Accessibility, 'a DEPwD empaneled auditor'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Verbatim from the live page</t>
-  </si>
-  <si>
-    <t xml:space="preserve">kotakneo.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kotak names no conformance standard or level</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Verbatim: 'recognised accessibility standards'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">'Kotak's statement is thin'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">It declares scope, names an auditor, states a phased roadmap, carries a Known Limitations section and a feedback route</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ungenerous. Article rewritten to credit it before noting gaps.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SEBI s.5.1 specifies IAAP; Pivotal is described as DEPwD-empanelled</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Both verbatim from their sources</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025/111 s.5.1; kotakneo.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Frame as a discrepancy, not as Pivotal being unqualified.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UTI AMC says it is 'progressively working towards enhancing digital accessibility in line with the WCAG'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Verbatim from the filed BRSR PDF, which carries independent assurance</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UTI/AMC/CS/SE/2026-27/0682, 24 Jun 2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">About a third of investor PDFs are untagged</t>
-  </si>
-  <si>
-    <t xml:space="preserve">25 of 76 PDFs hosted on the brokers' own domains lack a structure tree = 32.9%. Including third-party hosts it is 31 of 84 = 36.9%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">out/pdfcheck.json</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The article says 'from the brokers' own websites', so the 25/76 basis is the correct one. State the basis whenever the figure is used.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">'SEBI's own circular PDFs are tagged'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Three checked, all pass. Cannot generalise to all</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025/111, 2025/131, Dec 2025</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Article says 'the three I checked'.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">V1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vendors cite WCAG 2.1/2.2 AA, GIGW 3.0, IS 17802:2021</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Third party</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BarrierBreak readiness guide; enabled.in</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Live pages</t>
-  </si>
-  <si>
-    <t xml:space="preserve">V2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">'A seven-thousand-word readiness document'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Approximately 12,000-13,000 words</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Live page</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Corrected.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">V3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">'Still lists 31 July 2026, three weeks after it moved'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The page shows no publication or revision date at all, so no claim about when it was updated is available</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Corrected to 'as retrieved on 20 August 2026, it lists...'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">V4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">That guide lists the cancelled 14 Dec 2025 milestone as live</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Both sections confirmed on the live page</t>
-  </si>
-  <si>
-    <t xml:space="preserve">V5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">enabled.in advertises 'IAAP Certified' as a corporate credential</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Page text confirmed; IAAP certifies individuals, not companies</t>
-  </si>
-  <si>
-    <t xml:space="preserve">enabled.in</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Frame as a precision point, not an accusation.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">K1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">'Kotak has the lowest critical-violation density'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chat, 20 Aug</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Data</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OVERSTATED</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FALSE. Four brokers sit at 0.00/1k; Kotak is fifth at 0.21</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Broker Data tab</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Withdrawn. Never published.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">K2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">'Kotak has no failing charter PDFs'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MISLEADING. Kotak had zero charter PDFs tested; 0/0 is not a pass</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Same for Zerodha, HDFC and Dhan. Withdrawn.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">K3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kotak has the lowest serious-violation density</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.21 per 1,000 DOM nodes, lowest of ten</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Subject to S1 - unverified by hand.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">K4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kotak is the only broker with a published accessibility statement</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chat; article</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Link enumeration across ten home pages</t>
-  </si>
-  <si>
-    <t xml:space="preserve">K5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">'Kotak is best at nearly everything'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Two of the four supporting claims fail. What survives is K3 and K4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Withdrawn. Do not build a piece on it.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">K6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">'Disclosure does not predict artifact quality'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UNVERIFIED</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Spearman rho = 0.30, weakly positive. Band A has near-zero variance (7 of 10 score nil) so the correlation is not interpretable</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hypothesis not supported. Not publishable either way at n=10.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">K7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Band A cannot carry a scored article</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Range is 0/6 to 1/6; seven of ten score zero</t>
-  </si>
-  <si>
-    <t xml:space="preserve">K8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Band B has a fortyfold spread in serious-violation density</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.21 (Kotak) to 89.69 (Zerodha) per 1,000 DOM nodes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">X1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">This workbook's own first build</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Workbook</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Three errors found on review: it carried the un-normalised legacy-clause count (6, should be 7); it computed the untagged-PDF share on the wrong basis; and it counted 5paisa's unmeasured Band A as a zero</t>
-  </si>
-  <si>
-    <t xml:space="preserve">self-review</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The last is the exact error the rubric forbids -- scoring an unmeasured item as a failure. 5paisa now shows 'not measured'.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">All axe, reflow, text-spacing and focus-visibility results</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Not published</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Scan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No manual reproduction pass has been run</t>
-  </si>
-  <si>
-    <t xml:space="preserve">out/scan.json</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GATE: nothing from the scan may be published until each failure is reproduced by hand.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SUMMARY</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total claims</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Narrower than first stated</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Corrected</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Overstated / withdrawn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Not yet verified</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Failed verification (corrected + overstated)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Every 'Source' entry is a document retrieved and read in full, not a summary of it. Verified 20 August 2026.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rank</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Broker</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Band A score</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Band A max</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Grade</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Surfaces scanned</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Critical /1k DOM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Serious /1k DOM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total violation nodes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Worst surface</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Charter PDFs tested</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Charter PDFs failing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">All PDFs tested</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PDFs untagged</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Accessibility statement</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Groww</t>
-  </si>
-  <si>
-    <t xml:space="preserve">E</t>
-  </si>
-  <si>
-    <t xml:space="preserve">account_opening</t>
-  </si>
-  <si>
-    <t xml:space="preserve">no</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Zerodha</t>
-  </si>
-  <si>
-    <t xml:space="preserve">home</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Angel One</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D</t>
-  </si>
-  <si>
-    <t xml:space="preserve">grievance</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ICICI Securities</t>
-  </si>
-  <si>
-    <t xml:space="preserve">investor_charter</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Upstox</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kotak Securities</t>
-  </si>
-  <si>
-    <t xml:space="preserve">yes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HDFC Securities</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SBI Securities</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dhan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Motilal Oswal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5paisa</t>
-  </si>
-  <si>
-    <t xml:space="preserve">not measured</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOTALS / RANGE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Brokers in sample</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Brokers actually measured</t>
-  </si>
-  <si>
-    <t xml:space="preserve">With a published statement</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Band A scoring zero (of those measured)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Brokers at zero critical</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lowest serious /1k</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Highest serious /1k</t>
-  </si>
-  <si>
-    <t xml:space="preserve">All PDFs untagged</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WARNING: every Band B figure (columns G-I) is UNVERIFIED BY HAND -- see claim S1. Nothing here is publishable until each failure is manually reproduced.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Scan run 2026-08-20T02:50:13.406Z. 5paisa excluded from Band B: returns HTTP 403 to automated agents. No workaround attempted.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">'Charter PDFs tested = 0' means none were found, NOT that none failed. Zerodha, Kotak, HDFC and Dhan are 0/0.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5paisa is shown as 'not measured', never as zero. Scoring an unmeasured item as a failure is the error this project's rubric forbids.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Untagged-PDF share: 25 of 76 (32.9%) counting only PDFs on the brokers' own domains; 31 of 84 (36.9%) including third-party hosts. State the basis whenever quoting it.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Documents retrieved</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Characters of text</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Contains 'digital accessibility'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Legacy clause XVII</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Any 'accessib'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Any 'disab'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Corpus adequacy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">conclusive</t>
-  </si>
-  <si>
-    <t xml:space="preserve">thin - weak evidence</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NOT RETRIEVED</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Characters of charter text</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Carrying the digital accessibility right</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Carrying legacy clause XVII</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Conclusive corpora</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Method: each broker's charter page plus every charter-shaped PDF linked from it. Text whitespace-normalised before matching -- pdftotext line-wrapping broke a multi-word regex on the first run and undercounted clause XVII by one.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Circular number</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Date</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Effect</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Verification status</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Source used</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SEBI/HO/MIRSD/SECFATF/P/CIR/2025/74</t>
-  </si>
-  <si>
-    <t xml:space="preserve">23 May 2025</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Accessible digital KYC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NOT YET READ against primary text (OQ-3)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">nsdl.co.in mirror</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SEBI/HO/ITD-1/ITD_VIAP/P/CIR/2025/111</t>
-  </si>
-  <si>
-    <t xml:space="preserve">31 Jul 2025</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Base circular; Annexure I carries the substance</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Read in full</t>
-  </si>
-  <si>
-    <t xml:space="preserve">apmiindia.org mirror</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SEBI/HO/ITD-1/ITD_VIAP/P/CIR/2025/121</t>
-  </si>
-  <si>
-    <t xml:space="preserve">29 Aug 2025</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Extended all timelines; IA/RA reporting moved to BSE Ltd</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MUFG Intime mirror</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SEBI/HO/ITD-1/ITD_VIAP/P/CIR/2025/131</t>
-  </si>
-  <si>
-    <t xml:space="preserve">25 Sep 2025</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Compliance guidelines, Tables A-D, submission formats</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HO/13/19/13(2)2025-ITD-1_VIAP/I/187/2025</t>
-  </si>
-  <si>
-    <t xml:space="preserve">08 Dec 2025</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Replaced auditor milestone; Investor Charter right; SCORES</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HO/(411)2026-ITD-5_DIV2/I/17922/2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">31 Jul 2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Audit and remediation extended to 31 Oct 2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Read via reproducing notice</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BSE Notice 20260731-17</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sebi.gov.in is reachable with an explicit DNS resolve; the local resolver returns NXDOMAIN:  curl --resolve www.sebi.gov.in:443:202.191.181.158 https://www.sebi.gov.in/...</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mirrors are the exact SEBI PDFs redistributed by regulated market bodies under SEBI's supervision, not vendor summaries.</t>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>Claim</t>
+  </si>
+  <si>
+    <t>Where it appears</t>
+  </si>
+  <si>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Evidence</t>
+  </si>
+  <si>
+    <t>Source</t>
+  </si>
+  <si>
+    <t>Verified</t>
+  </si>
+  <si>
+    <t>Correction / note</t>
+  </si>
+  <si>
+    <t>R1</t>
+  </si>
+  <si>
+    <t>Supreme Court, 30 Apr 2025, held the right to digital access an intrinsic component of the right to life and personal liberty</t>
+  </si>
+  <si>
+    <t>Article; guide Ch.3</t>
+  </si>
+  <si>
+    <t>Regulation</t>
+  </si>
+  <si>
+    <t>VERIFIED</t>
+  </si>
+  <si>
+    <t>Quoted verbatim inside the circular itself</t>
+  </si>
+  <si>
+    <t>SEBI 2025/111 Annexure I s.A</t>
+  </si>
+  <si>
+    <t>2026-08-20</t>
+  </si>
+  <si>
+    <t>R2</t>
+  </si>
+  <si>
+    <t>The case is Pragya Prasun &amp; Ors. v. Union of India, heard with a Jain matter</t>
+  </si>
+  <si>
+    <t>Article; guide</t>
+  </si>
+  <si>
+    <t>NARROWER</t>
+  </si>
+  <si>
+    <t>Circular names 'Pragya Prasun &amp; Ors.' and 'Jain vs. Union of India'</t>
+  </si>
+  <si>
+    <t>First name 'Amar' comes from secondary coverage only. Article corrected to 'a Jain matter'.</t>
+  </si>
+  <si>
+    <t>R3</t>
+  </si>
+  <si>
+    <t>Standards are WCAG 2.1 or latest, GIGW latest, IS 17802, RPwD Act</t>
+  </si>
+  <si>
+    <t>Article; guide Ch.4</t>
+  </si>
+  <si>
+    <t>Verbatim, four numbered items</t>
+  </si>
+  <si>
+    <t>SEBI 2025/111 Annexure I s.B</t>
+  </si>
+  <si>
+    <t>R4</t>
+  </si>
+  <si>
+    <t>SEBI never writes WCAG 2.2, GIGW 3.0, or a year for IS 17802</t>
+  </si>
+  <si>
+    <t>Article</t>
+  </si>
+  <si>
+    <t>Full text of four circulars searched</t>
+  </si>
+  <si>
+    <t>2025/111, 2025/121, 2025/131, Dec 2025</t>
+  </si>
+  <si>
+    <t>R5</t>
+  </si>
+  <si>
+    <t>A Nodal Officer for digital accessibility is mandatory</t>
+  </si>
+  <si>
+    <t>Verbatim</t>
+  </si>
+  <si>
+    <t>2025/111 s.1.1-1.2</t>
+  </si>
+  <si>
+    <t>R6</t>
+  </si>
+  <si>
+    <t>An accessibility-specific grievance mechanism with escalation is required</t>
+  </si>
+  <si>
+    <t>2025/111 s.1.3</t>
+  </si>
+  <si>
+    <t>R7</t>
+  </si>
+  <si>
+    <t>Investor PDFs must follow accessible document standards; circular cites the WCAG PDF techniques</t>
+  </si>
+  <si>
+    <t>Verbatim, with the W3C URL</t>
+  </si>
+  <si>
+    <t>2025/111 s.2.2</t>
+  </si>
+  <si>
+    <t>R8</t>
+  </si>
+  <si>
+    <t>ISL, captions, descriptive audio and alt text are required</t>
+  </si>
+  <si>
+    <t>2025/111 s.2.1</t>
+  </si>
+  <si>
+    <t>R9</t>
+  </si>
+  <si>
+    <t>Audits must include usability testing by persons with disabilities</t>
+  </si>
+  <si>
+    <t>2025/111 s.5.1</t>
+  </si>
+  <si>
+    <t>R10</t>
+  </si>
+  <si>
+    <t>A disabled applicant may be rejected only after human review, with power to override automation</t>
+  </si>
+  <si>
+    <t>2025/111 s.4.2</t>
+  </si>
+  <si>
+    <t>R11</t>
+  </si>
+  <si>
+    <t>Responsibility for platform accessibility stays with the RE even for SaaS</t>
+  </si>
+  <si>
+    <t>The circular says 'responsibility', not 'liability'</t>
+  </si>
+  <si>
+    <t>2025/111 s.6.1</t>
+  </si>
+  <si>
+    <t>Article corrected: 'liability' replaced in two places.</t>
+  </si>
+  <si>
+    <t>R12</t>
+  </si>
+  <si>
+    <t>Audit and remediation deadline is 31 October 2026</t>
+  </si>
+  <si>
+    <t>Circular reproduced inside an exchange notice</t>
+  </si>
+  <si>
+    <t>HO/(411)2026-ITD-5_DIV2/I/17922/2026 via BSE Notice 20260731-17</t>
+  </si>
+  <si>
+    <t>R13</t>
+  </si>
+  <si>
+    <t>The 14 Dec 2025 auditor milestone was replaced, not supplemented</t>
+  </si>
+  <si>
+    <t>Verbatim: 'Instead of meeting the compliance requirement...'</t>
+  </si>
+  <si>
+    <t>Dec 2025 clarification para 3(a)</t>
+  </si>
+  <si>
+    <t>R14</t>
+  </si>
+  <si>
+    <t>Compliance is filed by email to SEBI, an exchange or a depository</t>
+  </si>
+  <si>
+    <t>Article; guide Ch.5</t>
+  </si>
+  <si>
+    <t>Submission mechanism and formats prescribed</t>
+  </si>
+  <si>
+    <t>2025/131 Part B; Dec 2025 Annexure A</t>
+  </si>
+  <si>
+    <t>R15</t>
+  </si>
+  <si>
+    <t>The circulars prescribe no penalty</t>
+  </si>
+  <si>
+    <t>Issued under s.11(1); no penalty clause in any circular read</t>
+  </si>
+  <si>
+    <t>All five read</t>
+  </si>
+  <si>
+    <t>Vendor claims of a penalty regime describe SEBI's general powers.</t>
+  </si>
+  <si>
+    <t>R16</t>
+  </si>
+  <si>
+    <t>'Six circulars'</t>
+  </si>
+  <si>
+    <t>Article v1</t>
+  </si>
+  <si>
+    <t>CORRECTED</t>
+  </si>
+  <si>
+    <t>SEBI's own Dec clarification references three prior circulars; the May 2025 KYC circular is a different series (MIRSD)</t>
+  </si>
+  <si>
+    <t>Dec 2025 clarification reference table</t>
+  </si>
+  <si>
+    <t>Corrected to: five digital accessibility circulars, preceded by a KYC circular.</t>
+  </si>
+  <si>
+    <t>R17</t>
+  </si>
+  <si>
+    <t>'Nothing in six circulars requires publication'</t>
+  </si>
+  <si>
+    <t>One of the six has not been read against primary text</t>
+  </si>
+  <si>
+    <t>OQ-3</t>
+  </si>
+  <si>
+    <t>Narrowed to the five actually read.</t>
+  </si>
+  <si>
+    <t>R18</t>
+  </si>
+  <si>
+    <t>24 obligations: 7 public, 4 artifact, 2 client, 11 not observable</t>
+  </si>
+  <si>
+    <t>Article; repo</t>
+  </si>
+  <si>
+    <t>Classification</t>
+  </si>
+  <si>
+    <t>Own classification, published in full</t>
+  </si>
+  <si>
+    <t>regulation/obligations.md</t>
+  </si>
+  <si>
+    <t>Presented as a classification, not a finding of fact. 7+4+2+11=24.</t>
+  </si>
+  <si>
+    <t>C1</t>
+  </si>
+  <si>
+    <t>SEBI's own Investor Charter contains no digital accessibility right</t>
+  </si>
+  <si>
+    <t>Charter</t>
+  </si>
+  <si>
+    <t>64,777 chars retrieved; zero matches for 'digital accessib' or 'disabilit'</t>
+  </si>
+  <si>
+    <t>investor.sebi.gov.in/Investor-charter.html</t>
+  </si>
+  <si>
+    <t>C2</t>
+  </si>
+  <si>
+    <t>The most recent Investor Charter circular for stock brokers is 21 Feb 2025</t>
+  </si>
+  <si>
+    <t>Circular located; Dec 2025 to May 2026 window not exhaustively searched</t>
+  </si>
+  <si>
+    <t>SEBI/HO/MIRSD/MIRSD-PoD1/P/CIR/2025/22</t>
+  </si>
+  <si>
+    <t>Keep the hedge 'that I can locate'. Tracked as OQ-1.</t>
+  </si>
+  <si>
+    <t>C3</t>
+  </si>
+  <si>
+    <t>'Eleven brokers' charters'</t>
+  </si>
+  <si>
+    <t>Ten. 5paisa returns HTTP 403 and no charter was retrievable</t>
+  </si>
+  <si>
+    <t>out/charter-verification.json</t>
+  </si>
+  <si>
+    <t>Corrected throughout the article.</t>
+  </si>
+  <si>
+    <t>C4</t>
+  </si>
+  <si>
+    <t>None of the charters checked contains the digital accessibility right</t>
+  </si>
+  <si>
+    <t>32 documents, 10 brokers, ~414,000 chars, whitespace-normalised. Zero matches</t>
+  </si>
+  <si>
+    <t>C5</t>
+  </si>
+  <si>
+    <t>'Every charter is the standard SEBI template, word for word'</t>
+  </si>
+  <si>
+    <t>Only 7 of 10 carry the legacy clause XVII</t>
+  </si>
+  <si>
+    <t>Removed; replaced with the claim actually evidenced.</t>
+  </si>
+  <si>
+    <t>C6</t>
+  </si>
+  <si>
+    <t>Corpus adequacy for two brokers</t>
+  </si>
+  <si>
+    <t>Kotak 2,728 chars and HDFC 5,874 are thin; likely landing pages not full charters</t>
+  </si>
+  <si>
+    <t>Stated as a caveat in the article.</t>
+  </si>
+  <si>
+    <t>C7</t>
+  </si>
+  <si>
+    <t>In Angel One's charter neither 'accessib' nor 'disab' appears</t>
+  </si>
+  <si>
+    <t>34,416 chars, neither string present</t>
+  </si>
+  <si>
+    <t>out/charters/angel-one.txt</t>
+  </si>
+  <si>
+    <t>D1</t>
+  </si>
+  <si>
+    <t>Of the brokers checked, one publishes an accessibility statement</t>
+  </si>
+  <si>
+    <t>Article; guide Ch.6</t>
+  </si>
+  <si>
+    <t>Disclosure</t>
+  </si>
+  <si>
+    <t>Kotak Securities; page retrieved and read in full</t>
+  </si>
+  <si>
+    <t>kotakneo.com/disclaimer/web-accessibility-statement/</t>
+  </si>
+  <si>
+    <t>D2</t>
+  </si>
+  <si>
+    <t>Kotak's statement names Pivotal Accessibility, 'a DEPwD empaneled auditor'</t>
+  </si>
+  <si>
+    <t>Verbatim from the live page</t>
+  </si>
+  <si>
+    <t>kotakneo.com</t>
+  </si>
+  <si>
+    <t>D3</t>
+  </si>
+  <si>
+    <t>Kotak names no conformance standard or level</t>
+  </si>
+  <si>
+    <t>Verbatim: 'recognised accessibility standards'</t>
+  </si>
+  <si>
+    <t>D4</t>
+  </si>
+  <si>
+    <t>'Kotak's statement is thin'</t>
+  </si>
+  <si>
+    <t>It declares scope, names an auditor, states a phased roadmap, carries a Known Limitations section and a feedback route</t>
+  </si>
+  <si>
+    <t>Ungenerous. Article rewritten to credit it before noting gaps.</t>
+  </si>
+  <si>
+    <t>D5</t>
+  </si>
+  <si>
+    <t>SEBI s.5.1 specifies IAAP; Pivotal is described as DEPwD-empanelled</t>
+  </si>
+  <si>
+    <t>Both verbatim from their sources</t>
+  </si>
+  <si>
+    <t>2025/111 s.5.1; kotakneo.com</t>
+  </si>
+  <si>
+    <t>Frame as a discrepancy, not as Pivotal being unqualified.</t>
+  </si>
+  <si>
+    <t>D6</t>
+  </si>
+  <si>
+    <t>UTI AMC says it is 'progressively working towards enhancing digital accessibility in line with the WCAG'</t>
+  </si>
+  <si>
+    <t>Verbatim from the filed BRSR PDF, which carries independent assurance</t>
+  </si>
+  <si>
+    <t>UTI/AMC/CS/SE/2026-27/0682, 24 Jun 2026</t>
+  </si>
+  <si>
+    <t>D7</t>
+  </si>
+  <si>
+    <t>About a third of investor PDFs are untagged</t>
+  </si>
+  <si>
+    <t>25 of 76 PDFs hosted on the brokers' own domains lack a structure tree = 32.9%. Including third-party hosts it is 31 of 84 = 36.9%</t>
+  </si>
+  <si>
+    <t>out/pdfcheck.json</t>
+  </si>
+  <si>
+    <t>The article says 'from the brokers' own websites', so the 25/76 basis is the correct one. State the basis whenever the figure is used.</t>
+  </si>
+  <si>
+    <t>D8</t>
+  </si>
+  <si>
+    <t>'SEBI's own circular PDFs are tagged'</t>
+  </si>
+  <si>
+    <t>Three checked, all pass. Cannot generalise to all</t>
+  </si>
+  <si>
+    <t>2025/111, 2025/131, Dec 2025</t>
+  </si>
+  <si>
+    <t>Article says 'the three I checked'.</t>
+  </si>
+  <si>
+    <t>V1</t>
+  </si>
+  <si>
+    <t>Vendors cite WCAG 2.1/2.2 AA, GIGW 3.0, IS 17802:2021</t>
+  </si>
+  <si>
+    <t>Third party</t>
+  </si>
+  <si>
+    <t>BarrierBreak readiness guide; enabled.in</t>
+  </si>
+  <si>
+    <t>Live pages</t>
+  </si>
+  <si>
+    <t>V2</t>
+  </si>
+  <si>
+    <t>'A seven-thousand-word readiness document'</t>
+  </si>
+  <si>
+    <t>Approximately 12,000-13,000 words</t>
+  </si>
+  <si>
+    <t>Live page</t>
+  </si>
+  <si>
+    <t>Corrected.</t>
+  </si>
+  <si>
+    <t>V3</t>
+  </si>
+  <si>
+    <t>'Still lists 31 July 2026, three weeks after it moved'</t>
+  </si>
+  <si>
+    <t>The page shows no publication or revision date at all, so no claim about when it was updated is available</t>
+  </si>
+  <si>
+    <t>Corrected to 'as retrieved on 20 August 2026, it lists...'</t>
+  </si>
+  <si>
+    <t>V4</t>
+  </si>
+  <si>
+    <t>That guide lists the cancelled 14 Dec 2025 milestone as live</t>
+  </si>
+  <si>
+    <t>Both sections confirmed on the live page</t>
+  </si>
+  <si>
+    <t>V5</t>
+  </si>
+  <si>
+    <t>enabled.in advertises 'IAAP Certified' as a corporate credential</t>
+  </si>
+  <si>
+    <t>Page text confirmed; IAAP certifies individuals, not companies</t>
+  </si>
+  <si>
+    <t>enabled.in</t>
+  </si>
+  <si>
+    <t>Frame as a precision point, not an accusation.</t>
+  </si>
+  <si>
+    <t>K1</t>
+  </si>
+  <si>
+    <t>'Kotak has the lowest critical-violation density'</t>
+  </si>
+  <si>
+    <t>Chat, 20 Aug</t>
+  </si>
+  <si>
+    <t>Data</t>
+  </si>
+  <si>
+    <t>OVERSTATED</t>
+  </si>
+  <si>
+    <t>FALSE. Four brokers sit at 0.00/1k; Kotak is fifth at 0.21</t>
+  </si>
+  <si>
+    <t>Broker Data tab</t>
+  </si>
+  <si>
+    <t>Withdrawn. Never published.</t>
+  </si>
+  <si>
+    <t>K2</t>
+  </si>
+  <si>
+    <t>'Kotak has no failing charter PDFs'</t>
+  </si>
+  <si>
+    <t>MISLEADING. Kotak had zero charter PDFs tested; 0/0 is not a pass</t>
+  </si>
+  <si>
+    <t>Same for Zerodha, HDFC and Dhan. Withdrawn.</t>
+  </si>
+  <si>
+    <t>K3</t>
+  </si>
+  <si>
+    <t>Kotak has the lowest serious-violation density</t>
+  </si>
+  <si>
+    <t>2.21 per 1,000 DOM nodes, lowest of ten</t>
+  </si>
+  <si>
+    <t>Subject to S1 - unverified by hand.</t>
+  </si>
+  <si>
+    <t>K4</t>
+  </si>
+  <si>
+    <t>Kotak is the only broker with a published accessibility statement</t>
+  </si>
+  <si>
+    <t>Chat; article</t>
+  </si>
+  <si>
+    <t>Link enumeration across ten home pages</t>
+  </si>
+  <si>
+    <t>K5</t>
+  </si>
+  <si>
+    <t>'Kotak is best at nearly everything'</t>
+  </si>
+  <si>
+    <t>Two of the four supporting claims fail. What survives is K3 and K4</t>
+  </si>
+  <si>
+    <t>Withdrawn. Do not build a piece on it.</t>
+  </si>
+  <si>
+    <t>K6</t>
+  </si>
+  <si>
+    <t>'Disclosure does not predict artifact quality'</t>
+  </si>
+  <si>
+    <t>UNVERIFIED</t>
+  </si>
+  <si>
+    <t>Spearman rho = 0.30, weakly positive. Band A has near-zero variance (7 of 10 score nil) so the correlation is not interpretable</t>
+  </si>
+  <si>
+    <t>Hypothesis not supported. Not publishable either way at n=10.</t>
+  </si>
+  <si>
+    <t>K7</t>
+  </si>
+  <si>
+    <t>Band A cannot carry a scored article</t>
+  </si>
+  <si>
+    <t>Range is 0/6 to 1/6; seven of ten score zero</t>
+  </si>
+  <si>
+    <t>K8</t>
+  </si>
+  <si>
+    <t>Band B has a fortyfold spread in serious-violation density</t>
+  </si>
+  <si>
+    <t>2.21 (Kotak) to 89.69 (Zerodha) per 1,000 DOM nodes</t>
+  </si>
+  <si>
+    <t>X1</t>
+  </si>
+  <si>
+    <t>This workbook's own first build</t>
+  </si>
+  <si>
+    <t>Workbook</t>
+  </si>
+  <si>
+    <t>Three errors found on review: it carried the un-normalised legacy-clause count (6, should be 7); it computed the untagged-PDF share on the wrong basis; and it counted 5paisa's unmeasured Band A as a zero</t>
+  </si>
+  <si>
+    <t>self-review</t>
+  </si>
+  <si>
+    <t>The last is the exact error the rubric forbids -- scoring an unmeasured item as a failure. 5paisa now shows 'not measured'.</t>
+  </si>
+  <si>
+    <t>S1</t>
+  </si>
+  <si>
+    <t>All axe, reflow, text-spacing and focus-visibility results</t>
+  </si>
+  <si>
+    <t>Not published</t>
+  </si>
+  <si>
+    <t>Scan</t>
+  </si>
+  <si>
+    <t>No manual reproduction pass has been run</t>
+  </si>
+  <si>
+    <t>out/scan.json</t>
+  </si>
+  <si>
+    <t>GATE: nothing from the scan may be published until each failure is reproduced by hand.</t>
+  </si>
+  <si>
+    <t>SUMMARY</t>
+  </si>
+  <si>
+    <t>Total claims</t>
+  </si>
+  <si>
+    <t>Narrower than first stated</t>
+  </si>
+  <si>
+    <t>Corrected</t>
+  </si>
+  <si>
+    <t>Overstated / withdrawn</t>
+  </si>
+  <si>
+    <t>Not yet verified</t>
+  </si>
+  <si>
+    <t>Failed verification (corrected + overstated)</t>
+  </si>
+  <si>
+    <t>Every 'Source' entry is a document retrieved and read in full, not a summary of it. Verified 20 August 2026.</t>
+  </si>
+  <si>
+    <t>Rank</t>
+  </si>
+  <si>
+    <t>Broker</t>
+  </si>
+  <si>
+    <t>Band A score</t>
+  </si>
+  <si>
+    <t>Band A max</t>
+  </si>
+  <si>
+    <t>Grade</t>
+  </si>
+  <si>
+    <t>Surfaces scanned</t>
+  </si>
+  <si>
+    <t>Critical /1k DOM</t>
+  </si>
+  <si>
+    <t>Serious /1k DOM</t>
+  </si>
+  <si>
+    <t>Total violation nodes</t>
+  </si>
+  <si>
+    <t>Worst surface</t>
+  </si>
+  <si>
+    <t>Charter PDFs tested</t>
+  </si>
+  <si>
+    <t>Charter PDFs failing</t>
+  </si>
+  <si>
+    <t>All PDFs tested</t>
+  </si>
+  <si>
+    <t>PDFs untagged</t>
+  </si>
+  <si>
+    <t>Accessibility statement</t>
+  </si>
+  <si>
+    <t>Groww</t>
+  </si>
+  <si>
+    <t>E</t>
+  </si>
+  <si>
+    <t>account_opening</t>
+  </si>
+  <si>
+    <t>no</t>
+  </si>
+  <si>
+    <t>Zerodha</t>
+  </si>
+  <si>
+    <t>home</t>
+  </si>
+  <si>
+    <t>Angel One</t>
+  </si>
+  <si>
+    <t>D</t>
+  </si>
+  <si>
+    <t>grievance</t>
+  </si>
+  <si>
+    <t>ICICI Securities</t>
+  </si>
+  <si>
+    <t>investor_charter</t>
+  </si>
+  <si>
+    <t>Upstox</t>
+  </si>
+  <si>
+    <t>Kotak Securities</t>
+  </si>
+  <si>
+    <t>yes</t>
+  </si>
+  <si>
+    <t>HDFC Securities</t>
+  </si>
+  <si>
+    <t>SBI Securities</t>
+  </si>
+  <si>
+    <t>Dhan</t>
+  </si>
+  <si>
+    <t>Motilal Oswal</t>
+  </si>
+  <si>
+    <t>5paisa</t>
+  </si>
+  <si>
+    <t>not measured</t>
+  </si>
+  <si>
+    <t>TOTALS / RANGE</t>
+  </si>
+  <si>
+    <t>Brokers in sample</t>
+  </si>
+  <si>
+    <t>Brokers actually measured</t>
+  </si>
+  <si>
+    <t>With a published statement</t>
+  </si>
+  <si>
+    <t>Band A scoring zero (of those measured)</t>
+  </si>
+  <si>
+    <t>Brokers at zero critical</t>
+  </si>
+  <si>
+    <t>Lowest serious /1k</t>
+  </si>
+  <si>
+    <t>Highest serious /1k</t>
+  </si>
+  <si>
+    <t>All PDFs untagged</t>
+  </si>
+  <si>
+    <t>WARNING: every Band B figure (columns G-I) is UNVERIFIED BY HAND -- see claim S1. Nothing here is publishable until each failure is manually reproduced.</t>
+  </si>
+  <si>
+    <t>Scan run 2026-08-20T02:50:13.406Z. 5paisa excluded from Band B: returns HTTP 403 to automated agents. No workaround attempted.</t>
+  </si>
+  <si>
+    <t>'Charter PDFs tested = 0' means none were found, NOT that none failed. Zerodha, Kotak, HDFC and Dhan are 0/0.</t>
+  </si>
+  <si>
+    <t>5paisa is shown as 'not measured', never as zero. Scoring an unmeasured item as a failure is the error this project's rubric forbids.</t>
+  </si>
+  <si>
+    <t>Untagged-PDF share: 25 of 76 (32.9%) counting only PDFs on the brokers' own domains; 31 of 84 (36.9%) including third-party hosts. State the basis whenever quoting it.</t>
+  </si>
+  <si>
+    <t>Documents retrieved</t>
+  </si>
+  <si>
+    <t>Characters of text</t>
+  </si>
+  <si>
+    <t>Contains 'digital accessibility'</t>
+  </si>
+  <si>
+    <t>Legacy clause XVII</t>
+  </si>
+  <si>
+    <t>Any 'accessib'</t>
+  </si>
+  <si>
+    <t>Any 'disab'</t>
+  </si>
+  <si>
+    <t>Corpus adequacy</t>
+  </si>
+  <si>
+    <t>conclusive</t>
+  </si>
+  <si>
+    <t>thin - weak evidence</t>
+  </si>
+  <si>
+    <t>NOT RETRIEVED</t>
+  </si>
+  <si>
+    <t>Characters of charter text</t>
+  </si>
+  <si>
+    <t>Carrying the digital accessibility right</t>
+  </si>
+  <si>
+    <t>Carrying legacy clause XVII</t>
+  </si>
+  <si>
+    <t>Conclusive corpora</t>
+  </si>
+  <si>
+    <t>Method: each broker's charter page plus every charter-shaped PDF linked from it. Text whitespace-normalised before matching -- pdftotext line-wrapping broke a multi-word regex on the first run and undercounted clause XVII by one.</t>
+  </si>
+  <si>
+    <t>#</t>
+  </si>
+  <si>
+    <t>Circular number</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Effect</t>
+  </si>
+  <si>
+    <t>Verification status</t>
+  </si>
+  <si>
+    <t>Source used</t>
+  </si>
+  <si>
+    <t>SEBI/HO/MIRSD/SECFATF/P/CIR/2025/74</t>
+  </si>
+  <si>
+    <t>23 May 2025</t>
+  </si>
+  <si>
+    <t>Accessible digital KYC</t>
+  </si>
+  <si>
+    <t>NOT YET READ against primary text (OQ-3)</t>
+  </si>
+  <si>
+    <t>nsdl.co.in mirror</t>
+  </si>
+  <si>
+    <t>SEBI/HO/ITD-1/ITD_VIAP/P/CIR/2025/111</t>
+  </si>
+  <si>
+    <t>31 Jul 2025</t>
+  </si>
+  <si>
+    <t>Base circular; Annexure I carries the substance</t>
+  </si>
+  <si>
+    <t>Read in full</t>
+  </si>
+  <si>
+    <t>apmiindia.org mirror</t>
+  </si>
+  <si>
+    <t>SEBI/HO/ITD-1/ITD_VIAP/P/CIR/2025/121</t>
+  </si>
+  <si>
+    <t>29 Aug 2025</t>
+  </si>
+  <si>
+    <t>Extended all timelines; IA/RA reporting moved to BSE Ltd</t>
+  </si>
+  <si>
+    <t>MUFG Intime mirror</t>
+  </si>
+  <si>
+    <t>SEBI/HO/ITD-1/ITD_VIAP/P/CIR/2025/131</t>
+  </si>
+  <si>
+    <t>25 Sep 2025</t>
+  </si>
+  <si>
+    <t>Compliance guidelines, Tables A-D, submission formats</t>
+  </si>
+  <si>
+    <t>HO/13/19/13(2)2025-ITD-1_VIAP/I/187/2025</t>
+  </si>
+  <si>
+    <t>08 Dec 2025</t>
+  </si>
+  <si>
+    <t>Replaced auditor milestone; Investor Charter right; SCORES</t>
+  </si>
+  <si>
+    <t>HO/(411)2026-ITD-5_DIV2/I/17922/2026</t>
+  </si>
+  <si>
+    <t>31 Jul 2026</t>
+  </si>
+  <si>
+    <t>Audit and remediation extended to 31 Oct 2026</t>
+  </si>
+  <si>
+    <t>Read via reproducing notice</t>
+  </si>
+  <si>
+    <t>BSE Notice 20260731-17</t>
+  </si>
+  <si>
+    <t>sebi.gov.in is reachable with an explicit DNS resolve; the local resolver returns NXDOMAIN:  curl --resolve www.sebi.gov.in:443:202.191.181.158 https://www.sebi.gov.in/...</t>
+  </si>
+  <si>
+    <t>Mirrors are the exact SEBI PDFs redistributed by regulated market bodies under SEBI's supervision, not vendor summaries.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="General"/>
-  </numFmts>
-  <fonts count="9">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1054,53 +1067,38 @@
     <font>
       <sz val="10"/>
       <name val="Arial"/>
-      <family val="0"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Arial"/>
-      <family val="0"/>
+      <family val="2"/>
     </font>
     <font>
+      <b/>
       <sz val="10"/>
       <name val="Arial"/>
-      <family val="0"/>
+      <family val="2"/>
     </font>
     <font>
-      <b val="true"/>
-      <sz val="10"/>
-      <color rgb="FFFFFFFF"/>
+      <i/>
+      <sz val="9"/>
       <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <i val="true"/>
-      <sz val="9"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <i val="true"/>
+      <i/>
       <sz val="9"/>
       <color rgb="FFC00000"/>
       <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="7">
@@ -1142,14 +1140,14 @@
     </fill>
   </fills>
   <borders count="2">
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left/>
       <right/>
       <top/>
@@ -1159,154 +1157,45 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="20">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </cellStyleXfs>
+  <cellXfs count="13">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-  </cellStyleXfs>
-  <cellXfs count="12">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="6">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="15" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
-    <cellStyle name="Currency" xfId="17" builtinId="4"/>
-    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
-    <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="8">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF1F3864"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFFFFF"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFD9D9D9"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF000000"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -1365,17 +1254,29 @@
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF333399"/>
       <rgbColor rgb="FF333333"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
     </indexedColors>
   </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -1417,12 +1318,12 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:minorFont>
@@ -1451,7 +1352,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="1"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -1472,7 +1373,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
@@ -1523,7 +1424,7 @@
           <a:path path="circle">
             <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
           </a:path>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -1541,33 +1442,32 @@
           <a:path path="circle">
             <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
           </a:path>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I60"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="58"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="52"/>
+    <col min="1" max="1" width="7" customWidth="1"/>
+    <col min="2" max="2" width="58" customWidth="1"/>
+    <col min="3" max="3" width="17" customWidth="1"/>
+    <col min="4" max="5" width="13" customWidth="1"/>
+    <col min="6" max="6" width="52" customWidth="1"/>
+    <col min="7" max="7" width="34" customWidth="1"/>
+    <col min="8" max="8" width="11" customWidth="1"/>
+    <col min="9" max="9" width="52" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1596,7 +1496,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>9</v>
       </c>
@@ -1623,7 +1523,7 @@
       </c>
       <c r="I2" s="3"/>
     </row>
-    <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>17</v>
       </c>
@@ -1652,7 +1552,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>23</v>
       </c>
@@ -1679,7 +1579,7 @@
       </c>
       <c r="I4" s="3"/>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>28</v>
       </c>
@@ -1706,7 +1606,7 @@
       </c>
       <c r="I5" s="3"/>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>33</v>
       </c>
@@ -1733,7 +1633,7 @@
       </c>
       <c r="I6" s="3"/>
     </row>
-    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>37</v>
       </c>
@@ -1760,7 +1660,7 @@
       </c>
       <c r="I7" s="3"/>
     </row>
-    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>40</v>
       </c>
@@ -1787,7 +1687,7 @@
       </c>
       <c r="I8" s="3"/>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>44</v>
       </c>
@@ -1814,7 +1714,7 @@
       </c>
       <c r="I9" s="3"/>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>47</v>
       </c>
@@ -1841,7 +1741,7 @@
       </c>
       <c r="I10" s="3"/>
     </row>
-    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
         <v>50</v>
       </c>
@@ -1868,7 +1768,7 @@
       </c>
       <c r="I11" s="3"/>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
         <v>53</v>
       </c>
@@ -1897,7 +1797,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
         <v>58</v>
       </c>
@@ -1924,7 +1824,7 @@
       </c>
       <c r="I13" s="3"/>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
         <v>62</v>
       </c>
@@ -1951,7 +1851,7 @@
       </c>
       <c r="I14" s="3"/>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
         <v>66</v>
       </c>
@@ -1978,7 +1878,7 @@
       </c>
       <c r="I15" s="3"/>
     </row>
-    <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
         <v>71</v>
       </c>
@@ -2007,7 +1907,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
         <v>76</v>
       </c>
@@ -2036,7 +1936,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
         <v>83</v>
       </c>
@@ -2065,7 +1965,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
         <v>88</v>
       </c>
@@ -2094,7 +1994,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
         <v>95</v>
       </c>
@@ -2121,7 +2021,7 @@
       </c>
       <c r="I20" s="3"/>
     </row>
-    <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
         <v>100</v>
       </c>
@@ -2150,7 +2050,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
         <v>105</v>
       </c>
@@ -2179,7 +2079,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
         <v>110</v>
       </c>
@@ -2206,7 +2106,7 @@
       </c>
       <c r="I23" s="3"/>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
         <v>113</v>
       </c>
@@ -2235,7 +2135,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
         <v>117</v>
       </c>
@@ -2264,7 +2164,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
         <v>121</v>
       </c>
@@ -2291,7 +2191,7 @@
       </c>
       <c r="I26" s="3"/>
     </row>
-    <row r="27" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
         <v>125</v>
       </c>
@@ -2310,7 +2210,7 @@
       <c r="F27" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="G27" s="3" t="s">
+      <c r="G27" s="12" t="s">
         <v>130</v>
       </c>
       <c r="H27" s="2" t="s">
@@ -2318,7 +2218,7 @@
       </c>
       <c r="I27" s="3"/>
     </row>
-    <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
         <v>131</v>
       </c>
@@ -2345,7 +2245,7 @@
       </c>
       <c r="I28" s="3"/>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A29" s="2" t="s">
         <v>135</v>
       </c>
@@ -2372,7 +2272,7 @@
       </c>
       <c r="I29" s="3"/>
     </row>
-    <row r="30" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A30" s="2" t="s">
         <v>138</v>
       </c>
@@ -2401,7 +2301,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A31" s="2" t="s">
         <v>142</v>
       </c>
@@ -2430,7 +2330,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
         <v>147</v>
       </c>
@@ -2449,7 +2349,7 @@
       <c r="F32" s="3" t="s">
         <v>149</v>
       </c>
-      <c r="G32" s="3" t="s">
+      <c r="G32" s="12" t="s">
         <v>150</v>
       </c>
       <c r="H32" s="2" t="s">
@@ -2457,7 +2357,7 @@
       </c>
       <c r="I32" s="3"/>
     </row>
-    <row r="33" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" spans="1:9" ht="42" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
         <v>151</v>
       </c>
@@ -2486,7 +2386,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A34" s="2" t="s">
         <v>156</v>
       </c>
@@ -2515,7 +2415,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A35" s="2" t="s">
         <v>161</v>
       </c>
@@ -2542,7 +2442,7 @@
       </c>
       <c r="I35" s="3"/>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A36" s="2" t="s">
         <v>166</v>
       </c>
@@ -2571,7 +2471,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A37" s="2" t="s">
         <v>171</v>
       </c>
@@ -2600,7 +2500,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A38" s="2" t="s">
         <v>175</v>
       </c>
@@ -2627,7 +2527,7 @@
       </c>
       <c r="I38" s="3"/>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A39" s="2" t="s">
         <v>178</v>
       </c>
@@ -2656,7 +2556,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A40" s="2" t="s">
         <v>183</v>
       </c>
@@ -2685,7 +2585,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="41" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A41" s="2" t="s">
         <v>191</v>
       </c>
@@ -2714,7 +2614,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A42" s="2" t="s">
         <v>195</v>
       </c>
@@ -2743,7 +2643,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A43" s="2" t="s">
         <v>199</v>
       </c>
@@ -2770,7 +2670,7 @@
       </c>
       <c r="I43" s="3"/>
     </row>
-    <row r="44" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="44" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A44" s="2" t="s">
         <v>203</v>
       </c>
@@ -2799,7 +2699,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="45" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A45" s="2" t="s">
         <v>207</v>
       </c>
@@ -2828,7 +2728,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="46" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A46" s="2" t="s">
         <v>212</v>
       </c>
@@ -2855,7 +2755,7 @@
       </c>
       <c r="I46" s="3"/>
     </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A47" s="2" t="s">
         <v>215</v>
       </c>
@@ -2884,7 +2784,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="48" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A48" s="2" t="s">
         <v>218</v>
       </c>
@@ -2910,7 +2810,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="49" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A49" s="2" t="s">
         <v>224</v>
       </c>
@@ -2939,115 +2839,106 @@
         <v>230</v>
       </c>
     </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="51" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A51" s="8" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="52" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A52" s="9" t="s">
         <v>232</v>
       </c>
-      <c r="B52" s="8" t="n">
-        <f aca="false">COUNTA(A2:A49)</f>
+      <c r="B52" s="8">
+        <f>COUNTA(A2:A49)</f>
         <v>48</v>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="53" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A53" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="B53" s="8" t="n">
-        <f aca="false">COUNTIF(E2:E49,"VERIFIED")</f>
+      <c r="B53" s="8">
+        <f>COUNTIF(E2:E49,"VERIFIED")</f>
         <v>30</v>
       </c>
     </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="54" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A54" s="9" t="s">
         <v>233</v>
       </c>
-      <c r="B54" s="8" t="n">
-        <f aca="false">COUNTIF(E2:E49,"NARROWER")</f>
+      <c r="B54" s="8">
+        <f>COUNTIF(E2:E49,"NARROWER")</f>
         <v>5</v>
       </c>
     </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="55" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A55" s="9" t="s">
         <v>234</v>
       </c>
-      <c r="B55" s="8" t="n">
-        <f aca="false">COUNTIF(E2:E49,"CORRECTED")</f>
+      <c r="B55" s="8">
+        <f>COUNTIF(E2:E49,"CORRECTED")</f>
         <v>7</v>
       </c>
     </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="56" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A56" s="9" t="s">
         <v>235</v>
       </c>
-      <c r="B56" s="8" t="n">
-        <f aca="false">COUNTIF(E2:E49,"OVERSTATED")</f>
+      <c r="B56" s="8">
+        <f>COUNTIF(E2:E49,"OVERSTATED")</f>
         <v>3</v>
       </c>
     </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="57" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A57" s="9" t="s">
         <v>236</v>
       </c>
-      <c r="B57" s="8" t="n">
-        <f aca="false">COUNTIF(E2:E49,"UNVERIFIED")</f>
+      <c r="B57" s="8">
+        <f>COUNTIF(E2:E49,"UNVERIFIED")</f>
         <v>2</v>
       </c>
     </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="58" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A58" s="9" t="s">
         <v>237</v>
       </c>
-      <c r="B58" s="8" t="n">
-        <f aca="false">COUNTIF(E2:E49,"CORRECTED")+COUNTIF(E2:E49,"OVERSTATED")</f>
+      <c r="B58" s="8">
+        <f>COUNTIF(E2:E49,"CORRECTED")+COUNTIF(E2:E49,"OVERSTATED")</f>
         <v>10</v>
       </c>
     </row>
-    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="60" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A60" s="10" t="s">
         <v>238</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I49"/>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <autoFilter ref="A1:I49" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
-  <drawing r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:O31"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="11" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="13" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="14"/>
+    <col min="1" max="1" width="6" customWidth="1"/>
+    <col min="2" max="2" width="20" customWidth="1"/>
+    <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="4" max="4" width="11" customWidth="1"/>
+    <col min="5" max="5" width="8" customWidth="1"/>
+    <col min="6" max="6" width="11" customWidth="1"/>
+    <col min="7" max="8" width="12" customWidth="1"/>
+    <col min="9" max="9" width="13" customWidth="1"/>
+    <col min="10" max="10" width="17" customWidth="1"/>
+    <col min="11" max="12" width="12" customWidth="1"/>
+    <col min="13" max="14" width="11" customWidth="1"/>
+    <col min="15" max="15" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:15" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>239</v>
       </c>
@@ -3094,478 +2985,478 @@
         <v>253</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="n">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A2" s="2">
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>254</v>
       </c>
-      <c r="C2" s="2" t="n">
+      <c r="C2" s="2">
         <v>0</v>
       </c>
-      <c r="D2" s="2" t="n">
+      <c r="D2" s="2">
         <v>6</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>255</v>
       </c>
-      <c r="F2" s="2" t="n">
+      <c r="F2" s="2">
         <v>4</v>
       </c>
-      <c r="G2" s="2" t="n">
+      <c r="G2" s="2">
         <v>0</v>
       </c>
-      <c r="H2" s="2" t="n">
+      <c r="H2" s="2">
         <v>43.44</v>
       </c>
-      <c r="I2" s="2" t="n">
+      <c r="I2" s="2">
         <v>328</v>
       </c>
       <c r="J2" s="2" t="s">
         <v>256</v>
       </c>
-      <c r="K2" s="2" t="n">
+      <c r="K2" s="2">
         <v>4</v>
       </c>
-      <c r="L2" s="2" t="n">
+      <c r="L2" s="2">
         <v>1</v>
       </c>
-      <c r="M2" s="2" t="n">
+      <c r="M2" s="2">
         <v>14</v>
       </c>
-      <c r="N2" s="2" t="n">
+      <c r="N2" s="2">
         <v>3</v>
       </c>
       <c r="O2" s="2" t="s">
         <v>257</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="n">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A3" s="2">
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>258</v>
       </c>
-      <c r="C3" s="2" t="n">
+      <c r="C3" s="2">
         <v>0</v>
       </c>
-      <c r="D3" s="2" t="n">
+      <c r="D3" s="2">
         <v>5</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>255</v>
       </c>
-      <c r="F3" s="2" t="n">
+      <c r="F3" s="2">
         <v>5</v>
       </c>
-      <c r="G3" s="2" t="n">
+      <c r="G3" s="2">
         <v>0.52</v>
       </c>
-      <c r="H3" s="2" t="n">
+      <c r="H3" s="2">
         <v>89.69</v>
       </c>
-      <c r="I3" s="2" t="n">
+      <c r="I3" s="2">
         <v>231</v>
       </c>
       <c r="J3" s="2" t="s">
         <v>259</v>
       </c>
-      <c r="K3" s="2" t="n">
+      <c r="K3" s="2">
         <v>0</v>
       </c>
-      <c r="L3" s="2" t="n">
+      <c r="L3" s="2">
         <v>0</v>
       </c>
-      <c r="M3" s="2" t="n">
+      <c r="M3" s="2">
         <v>0</v>
       </c>
-      <c r="N3" s="2" t="n">
+      <c r="N3" s="2">
         <v>0</v>
       </c>
       <c r="O3" s="2" t="s">
         <v>257</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="n">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A4" s="2">
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>260</v>
       </c>
-      <c r="C4" s="2" t="n">
+      <c r="C4" s="2">
         <v>1</v>
       </c>
-      <c r="D4" s="2" t="n">
+      <c r="D4" s="2">
         <v>6</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="F4" s="2" t="n">
+      <c r="F4" s="2">
         <v>5</v>
       </c>
-      <c r="G4" s="2" t="n">
+      <c r="G4" s="2">
         <v>1.96</v>
       </c>
-      <c r="H4" s="2" t="n">
+      <c r="H4" s="2">
         <v>4.08</v>
       </c>
-      <c r="I4" s="2" t="n">
+      <c r="I4" s="2">
         <v>51</v>
       </c>
       <c r="J4" s="2" t="s">
         <v>262</v>
       </c>
-      <c r="K4" s="2" t="n">
+      <c r="K4" s="2">
         <v>4</v>
       </c>
-      <c r="L4" s="2" t="n">
+      <c r="L4" s="2">
         <v>0</v>
       </c>
-      <c r="M4" s="2" t="n">
+      <c r="M4" s="2">
         <v>9</v>
       </c>
-      <c r="N4" s="2" t="n">
+      <c r="N4" s="2">
         <v>1</v>
       </c>
       <c r="O4" s="2" t="s">
         <v>257</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="n">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A5" s="2">
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>263</v>
       </c>
-      <c r="C5" s="2" t="n">
+      <c r="C5" s="2">
         <v>0</v>
       </c>
-      <c r="D5" s="2" t="n">
+      <c r="D5" s="2">
         <v>6</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>255</v>
       </c>
-      <c r="F5" s="2" t="n">
+      <c r="F5" s="2">
         <v>3</v>
       </c>
-      <c r="G5" s="2" t="n">
+      <c r="G5" s="2">
         <v>0.88</v>
       </c>
-      <c r="H5" s="2" t="n">
+      <c r="H5" s="2">
         <v>77.23</v>
       </c>
-      <c r="I5" s="2" t="n">
+      <c r="I5" s="2">
         <v>243</v>
       </c>
       <c r="J5" s="2" t="s">
         <v>264</v>
       </c>
-      <c r="K5" s="2" t="n">
+      <c r="K5" s="2">
         <v>4</v>
       </c>
-      <c r="L5" s="2" t="n">
+      <c r="L5" s="2">
         <v>1</v>
       </c>
-      <c r="M5" s="2" t="n">
+      <c r="M5" s="2">
         <v>12</v>
       </c>
-      <c r="N5" s="2" t="n">
+      <c r="N5" s="2">
         <v>6</v>
       </c>
       <c r="O5" s="2" t="s">
         <v>257</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="n">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A6" s="2">
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>265</v>
       </c>
-      <c r="C6" s="2" t="n">
+      <c r="C6" s="2">
         <v>0</v>
       </c>
-      <c r="D6" s="2" t="n">
+      <c r="D6" s="2">
         <v>6</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>255</v>
       </c>
-      <c r="F6" s="2" t="n">
+      <c r="F6" s="2">
         <v>4</v>
       </c>
-      <c r="G6" s="2" t="n">
+      <c r="G6" s="2">
         <v>0</v>
       </c>
-      <c r="H6" s="2" t="n">
+      <c r="H6" s="2">
         <v>3.98</v>
       </c>
-      <c r="I6" s="2" t="n">
+      <c r="I6" s="2">
         <v>22</v>
       </c>
       <c r="J6" s="2" t="s">
         <v>259</v>
       </c>
-      <c r="K6" s="2" t="n">
+      <c r="K6" s="2">
         <v>2</v>
       </c>
-      <c r="L6" s="2" t="n">
+      <c r="L6" s="2">
         <v>2</v>
       </c>
-      <c r="M6" s="2" t="n">
+      <c r="M6" s="2">
         <v>11</v>
       </c>
-      <c r="N6" s="2" t="n">
+      <c r="N6" s="2">
         <v>4</v>
       </c>
       <c r="O6" s="2" t="s">
         <v>257</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="n">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A7" s="2">
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>266</v>
       </c>
-      <c r="C7" s="2" t="n">
+      <c r="C7" s="2">
         <v>1</v>
       </c>
-      <c r="D7" s="2" t="n">
+      <c r="D7" s="2">
         <v>5</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="F7" s="2" t="n">
+      <c r="F7" s="2">
         <v>6</v>
       </c>
-      <c r="G7" s="2" t="n">
+      <c r="G7" s="2">
         <v>0.21</v>
       </c>
-      <c r="H7" s="2" t="n">
+      <c r="H7" s="2">
         <v>2.21</v>
       </c>
-      <c r="I7" s="2" t="n">
+      <c r="I7" s="2">
         <v>44</v>
       </c>
       <c r="J7" s="2" t="s">
         <v>256</v>
       </c>
-      <c r="K7" s="2" t="n">
+      <c r="K7" s="2">
         <v>0</v>
       </c>
-      <c r="L7" s="2" t="n">
+      <c r="L7" s="2">
         <v>0</v>
       </c>
-      <c r="M7" s="2" t="n">
+      <c r="M7" s="2">
         <v>4</v>
       </c>
-      <c r="N7" s="2" t="n">
+      <c r="N7" s="2">
         <v>2</v>
       </c>
       <c r="O7" s="2" t="s">
         <v>267</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="n">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A8" s="2">
         <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>268</v>
       </c>
-      <c r="C8" s="2" t="n">
+      <c r="C8" s="2">
         <v>0</v>
       </c>
-      <c r="D8" s="2" t="n">
+      <c r="D8" s="2">
         <v>5</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>255</v>
       </c>
-      <c r="F8" s="2" t="n">
+      <c r="F8" s="2">
         <v>4</v>
       </c>
-      <c r="G8" s="2" t="n">
+      <c r="G8" s="2">
         <v>1.83</v>
       </c>
-      <c r="H8" s="2" t="n">
+      <c r="H8" s="2">
         <v>4.79</v>
       </c>
-      <c r="I8" s="2" t="n">
+      <c r="I8" s="2">
         <v>41</v>
       </c>
       <c r="J8" s="2" t="s">
         <v>259</v>
       </c>
-      <c r="K8" s="2" t="n">
+      <c r="K8" s="2">
         <v>0</v>
       </c>
-      <c r="L8" s="2" t="n">
+      <c r="L8" s="2">
         <v>0</v>
       </c>
-      <c r="M8" s="2" t="n">
+      <c r="M8" s="2">
         <v>3</v>
       </c>
-      <c r="N8" s="2" t="n">
+      <c r="N8" s="2">
         <v>3</v>
       </c>
       <c r="O8" s="2" t="s">
         <v>257</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="n">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A9" s="2">
         <v>8</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>269</v>
       </c>
-      <c r="C9" s="2" t="n">
+      <c r="C9" s="2">
         <v>1</v>
       </c>
-      <c r="D9" s="2" t="n">
+      <c r="D9" s="2">
         <v>6</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="F9" s="2" t="n">
+      <c r="F9" s="2">
         <v>3</v>
       </c>
-      <c r="G9" s="2" t="n">
+      <c r="G9" s="2">
         <v>0</v>
       </c>
-      <c r="H9" s="2" t="n">
-        <v>9.62</v>
-      </c>
-      <c r="I9" s="2" t="n">
+      <c r="H9" s="2">
+        <v>9.6199999999999992</v>
+      </c>
+      <c r="I9" s="2">
         <v>39</v>
       </c>
       <c r="J9" s="2" t="s">
         <v>259</v>
       </c>
-      <c r="K9" s="2" t="n">
+      <c r="K9" s="2">
         <v>3</v>
       </c>
-      <c r="L9" s="2" t="n">
+      <c r="L9" s="2">
         <v>0</v>
       </c>
-      <c r="M9" s="2" t="n">
+      <c r="M9" s="2">
         <v>9</v>
       </c>
-      <c r="N9" s="2" t="n">
+      <c r="N9" s="2">
         <v>1</v>
       </c>
       <c r="O9" s="2" t="s">
         <v>257</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2" t="n">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A10" s="2">
         <v>9</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>270</v>
       </c>
-      <c r="C10" s="2" t="n">
+      <c r="C10" s="2">
         <v>0</v>
       </c>
-      <c r="D10" s="2" t="n">
+      <c r="D10" s="2">
         <v>5</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>255</v>
       </c>
-      <c r="F10" s="2" t="n">
+      <c r="F10" s="2">
         <v>5</v>
       </c>
-      <c r="G10" s="2" t="n">
+      <c r="G10" s="2">
         <v>1.58</v>
       </c>
-      <c r="H10" s="2" t="n">
+      <c r="H10" s="2">
         <v>29.21</v>
       </c>
-      <c r="I10" s="2" t="n">
+      <c r="I10" s="2">
         <v>353</v>
       </c>
       <c r="J10" s="2" t="s">
         <v>256</v>
       </c>
-      <c r="K10" s="2" t="n">
+      <c r="K10" s="2">
         <v>0</v>
       </c>
-      <c r="L10" s="2" t="n">
+      <c r="L10" s="2">
         <v>0</v>
       </c>
-      <c r="M10" s="2" t="n">
+      <c r="M10" s="2">
         <v>9</v>
       </c>
-      <c r="N10" s="2" t="n">
+      <c r="N10" s="2">
         <v>3</v>
       </c>
       <c r="O10" s="2" t="s">
         <v>257</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="n">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A11" s="2">
         <v>10</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>271</v>
       </c>
-      <c r="C11" s="2" t="n">
+      <c r="C11" s="2">
         <v>0</v>
       </c>
-      <c r="D11" s="2" t="n">
+      <c r="D11" s="2">
         <v>6</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>255</v>
       </c>
-      <c r="F11" s="2" t="n">
+      <c r="F11" s="2">
         <v>3</v>
       </c>
-      <c r="G11" s="2" t="n">
+      <c r="G11" s="2">
         <v>0</v>
       </c>
-      <c r="H11" s="2" t="n">
+      <c r="H11" s="2">
         <v>12.92</v>
       </c>
-      <c r="I11" s="2" t="n">
+      <c r="I11" s="2">
         <v>50</v>
       </c>
       <c r="J11" s="2" t="s">
         <v>256</v>
       </c>
-      <c r="K11" s="2" t="n">
+      <c r="K11" s="2">
         <v>3</v>
       </c>
-      <c r="L11" s="2" t="n">
+      <c r="L11" s="2">
         <v>3</v>
       </c>
-      <c r="M11" s="2" t="n">
+      <c r="M11" s="2">
         <v>5</v>
       </c>
-      <c r="N11" s="2" t="n">
+      <c r="N11" s="2">
         <v>2</v>
       </c>
       <c r="O11" s="2" t="s">
         <v>257</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2" t="n">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A12" s="2">
         <v>11</v>
       </c>
       <c r="B12" s="2" t="s">
@@ -3580,7 +3471,7 @@
       <c r="E12" s="2" t="s">
         <v>273</v>
       </c>
-      <c r="F12" s="2" t="n">
+      <c r="F12" s="2">
         <v>0</v>
       </c>
       <c r="G12" s="2" t="s">
@@ -3595,182 +3486,174 @@
       <c r="J12" s="2" t="s">
         <v>273</v>
       </c>
-      <c r="K12" s="2" t="n">
+      <c r="K12" s="2">
         <v>0</v>
       </c>
-      <c r="L12" s="2" t="n">
+      <c r="L12" s="2">
         <v>0</v>
       </c>
-      <c r="M12" s="2" t="n">
+      <c r="M12" s="2">
         <v>0</v>
       </c>
-      <c r="N12" s="2" t="n">
+      <c r="N12" s="2">
         <v>0</v>
       </c>
       <c r="O12" s="2" t="s">
         <v>257</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
       <c r="B14" s="8" t="s">
         <v>274</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
       <c r="B15" s="9" t="s">
         <v>275</v>
       </c>
-      <c r="C15" s="8" t="n">
-        <f aca="false">COUNTA(B2:B12)</f>
+      <c r="C15" s="8">
+        <f>COUNTA(B2:B12)</f>
         <v>11</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
       <c r="B16" s="9" t="s">
         <v>276</v>
       </c>
-      <c r="C16" s="8" t="n">
-        <f aca="false">COUNTA(B2:B12)-COUNTIF(C2:C12,"not measured")</f>
+      <c r="C16" s="8">
+        <f>COUNTA(B2:B12)-COUNTIF(C2:C12,"not measured")</f>
         <v>10</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B17" s="9" t="s">
         <v>277</v>
       </c>
-      <c r="C17" s="8" t="n">
-        <f aca="false">COUNTIF(O2:O12,"yes")</f>
+      <c r="C17" s="8">
+        <f>COUNTIF(O2:O12,"yes")</f>
         <v>1</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B18" s="9" t="s">
         <v>278</v>
       </c>
-      <c r="C18" s="8" t="n">
-        <f aca="false">COUNTIF(C2:C12,0)</f>
+      <c r="C18" s="8">
+        <f>COUNTIF(C2:C12,0)</f>
         <v>7</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B19" s="9" t="s">
         <v>279</v>
       </c>
-      <c r="C19" s="8" t="n">
-        <f aca="false">COUNTIF(G2:G12,0)</f>
+      <c r="C19" s="8">
+        <f>COUNTIF(G2:G12,0)</f>
         <v>4</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B20" s="9" t="s">
         <v>280</v>
       </c>
-      <c r="C20" s="8" t="n">
-        <f aca="false">MIN(H2:H12)</f>
+      <c r="C20" s="8">
+        <f>MIN(H2:H12)</f>
         <v>2.21</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B21" s="9" t="s">
         <v>281</v>
       </c>
-      <c r="C21" s="8" t="n">
-        <f aca="false">MAX(H2:H12)</f>
+      <c r="C21" s="8">
+        <f>MAX(H2:H12)</f>
         <v>89.69</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B22" s="9" t="s">
         <v>250</v>
       </c>
-      <c r="C22" s="8" t="n">
-        <f aca="false">SUM(L2:L12)</f>
+      <c r="C22" s="8">
+        <f>SUM(L2:L12)</f>
         <v>7</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B23" s="9" t="s">
         <v>249</v>
       </c>
-      <c r="C23" s="8" t="n">
-        <f aca="false">SUM(K2:K12)</f>
+      <c r="C23" s="8">
+        <f>SUM(K2:K12)</f>
         <v>20</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B24" s="9" t="s">
         <v>282</v>
       </c>
-      <c r="C24" s="8" t="n">
-        <f aca="false">SUM(N2:N12)</f>
+      <c r="C24" s="8">
+        <f>SUM(N2:N12)</f>
         <v>25</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B25" s="9" t="s">
         <v>251</v>
       </c>
-      <c r="C25" s="8" t="n">
-        <f aca="false">SUM(M2:M12)</f>
+      <c r="C25" s="8">
+        <f>SUM(M2:M12)</f>
         <v>76</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B27" s="11" t="s">
         <v>283</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B28" s="10" t="s">
         <v>284</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B29" s="11" t="s">
         <v>285</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B30" s="11" t="s">
         <v>286</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="31" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B31" s="10" t="s">
         <v>287</v>
       </c>
     </row>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:I21"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="22"/>
+    <col min="1" max="1" width="6" customWidth="1"/>
+    <col min="2" max="2" width="20" customWidth="1"/>
+    <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="4" max="4" width="13" customWidth="1"/>
+    <col min="5" max="5" width="15" customWidth="1"/>
+    <col min="6" max="6" width="12" customWidth="1"/>
+    <col min="7" max="7" width="11" customWidth="1"/>
+    <col min="8" max="8" width="10" customWidth="1"/>
+    <col min="9" max="9" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>239</v>
       </c>
@@ -3799,17 +3682,17 @@
         <v>294</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="n">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A2" s="2">
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>254</v>
       </c>
-      <c r="C2" s="2" t="n">
+      <c r="C2" s="2">
         <v>5</v>
       </c>
-      <c r="D2" s="2" t="n">
+      <c r="D2" s="2">
         <v>91533</v>
       </c>
       <c r="E2" s="2" t="s">
@@ -3828,17 +3711,17 @@
         <v>295</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="n">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A3" s="2">
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>258</v>
       </c>
-      <c r="C3" s="2" t="n">
+      <c r="C3" s="2">
         <v>1</v>
       </c>
-      <c r="D3" s="2" t="n">
+      <c r="D3" s="2">
         <v>22183</v>
       </c>
       <c r="E3" s="2" t="s">
@@ -3857,17 +3740,17 @@
         <v>295</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="n">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A4" s="2">
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>260</v>
       </c>
-      <c r="C4" s="2" t="n">
+      <c r="C4" s="2">
         <v>5</v>
       </c>
-      <c r="D4" s="2" t="n">
+      <c r="D4" s="2">
         <v>34416</v>
       </c>
       <c r="E4" s="2" t="s">
@@ -3886,17 +3769,17 @@
         <v>295</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="n">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A5" s="2">
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>263</v>
       </c>
-      <c r="C5" s="2" t="n">
+      <c r="C5" s="2">
         <v>5</v>
       </c>
-      <c r="D5" s="2" t="n">
+      <c r="D5" s="2">
         <v>49058</v>
       </c>
       <c r="E5" s="2" t="s">
@@ -3915,17 +3798,17 @@
         <v>295</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="n">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A6" s="2">
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>265</v>
       </c>
-      <c r="C6" s="2" t="n">
+      <c r="C6" s="2">
         <v>3</v>
       </c>
-      <c r="D6" s="2" t="n">
+      <c r="D6" s="2">
         <v>52670</v>
       </c>
       <c r="E6" s="2" t="s">
@@ -3944,17 +3827,17 @@
         <v>295</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="n">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A7" s="2">
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>266</v>
       </c>
-      <c r="C7" s="2" t="n">
+      <c r="C7" s="2">
         <v>1</v>
       </c>
-      <c r="D7" s="2" t="n">
+      <c r="D7" s="2">
         <v>2728</v>
       </c>
       <c r="E7" s="2" t="s">
@@ -3973,17 +3856,17 @@
         <v>296</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="n">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A8" s="2">
         <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>268</v>
       </c>
-      <c r="C8" s="2" t="n">
+      <c r="C8" s="2">
         <v>1</v>
       </c>
-      <c r="D8" s="2" t="n">
+      <c r="D8" s="2">
         <v>5874</v>
       </c>
       <c r="E8" s="2" t="s">
@@ -4002,17 +3885,17 @@
         <v>296</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="n">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A9" s="2">
         <v>8</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>269</v>
       </c>
-      <c r="C9" s="2" t="n">
+      <c r="C9" s="2">
         <v>4</v>
       </c>
-      <c r="D9" s="2" t="n">
+      <c r="D9" s="2">
         <v>43250</v>
       </c>
       <c r="E9" s="2" t="s">
@@ -4031,17 +3914,17 @@
         <v>295</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2" t="n">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A10" s="2">
         <v>9</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>270</v>
       </c>
-      <c r="C10" s="2" t="n">
+      <c r="C10" s="2">
         <v>3</v>
       </c>
-      <c r="D10" s="2" t="n">
+      <c r="D10" s="2">
         <v>71436</v>
       </c>
       <c r="E10" s="2" t="s">
@@ -4060,17 +3943,17 @@
         <v>295</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="n">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A11" s="2">
         <v>10</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>271</v>
       </c>
-      <c r="C11" s="2" t="n">
+      <c r="C11" s="2">
         <v>4</v>
       </c>
-      <c r="D11" s="2" t="n">
+      <c r="D11" s="2">
         <v>44057</v>
       </c>
       <c r="E11" s="2" t="s">
@@ -4089,17 +3972,17 @@
         <v>295</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2" t="n">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A12" s="2">
         <v>11</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>272</v>
       </c>
-      <c r="C12" s="2" t="n">
+      <c r="C12" s="2">
         <v>0</v>
       </c>
-      <c r="D12" s="2" t="n">
+      <c r="D12" s="2">
         <v>0</v>
       </c>
       <c r="E12" s="2" t="s">
@@ -4118,84 +4001,76 @@
         <v>297</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B14" s="9" t="s">
         <v>288</v>
       </c>
-      <c r="C14" s="8" t="n">
-        <f aca="false">SUM(C2:C12)</f>
+      <c r="C14" s="8">
+        <f>SUM(C2:C12)</f>
         <v>32</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B15" s="9" t="s">
         <v>298</v>
       </c>
-      <c r="C15" s="8" t="n">
-        <f aca="false">SUM(D2:D12)</f>
+      <c r="C15" s="8">
+        <f>SUM(D2:D12)</f>
         <v>417205</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B16" s="9" t="s">
         <v>299</v>
       </c>
-      <c r="C16" s="8" t="n">
-        <f aca="false">COUNTIF(E2:E12,"YES")</f>
+      <c r="C16" s="8">
+        <f>COUNTIF(E2:E12,"YES")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B17" s="9" t="s">
         <v>300</v>
       </c>
-      <c r="C17" s="8" t="n">
-        <f aca="false">COUNTIF(F2:F12,"yes")</f>
+      <c r="C17" s="8">
+        <f>COUNTIF(F2:F12,"yes")</f>
         <v>7</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B18" s="9" t="s">
         <v>301</v>
       </c>
-      <c r="C18" s="8" t="n">
-        <f aca="false">COUNTIF(I2:I12,"conclusive")</f>
+      <c r="C18" s="8">
+        <f>COUNTIF(I2:I12,"conclusive")</f>
         <v>8</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B21" s="10" t="s">
         <v>302</v>
       </c>
     </row>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:F10"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="50"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="26"/>
+    <col min="1" max="1" width="4" customWidth="1"/>
+    <col min="2" max="2" width="40" customWidth="1"/>
+    <col min="3" max="3" width="13" customWidth="1"/>
+    <col min="4" max="4" width="50" customWidth="1"/>
+    <col min="5" max="5" width="34" customWidth="1"/>
+    <col min="6" max="6" width="26" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>303</v>
       </c>
@@ -4215,8 +4090,8 @@
         <v>308</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="n">
+    <row r="2" spans="1:6" ht="28" x14ac:dyDescent="0.2">
+      <c r="A2" s="2">
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
@@ -4235,8 +4110,8 @@
         <v>313</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="n">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A3" s="2">
         <v>2</v>
       </c>
       <c r="B3" s="3" t="s">
@@ -4255,8 +4130,8 @@
         <v>318</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="n">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A4" s="2">
         <v>3</v>
       </c>
       <c r="B4" s="3" t="s">
@@ -4275,8 +4150,8 @@
         <v>322</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="n">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A5" s="2">
         <v>4</v>
       </c>
       <c r="B5" s="3" t="s">
@@ -4295,8 +4170,8 @@
         <v>318</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="n">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A6" s="2">
         <v>5</v>
       </c>
       <c r="B6" s="3" t="s">
@@ -4315,8 +4190,8 @@
         <v>318</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="n">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A7" s="2">
         <v>6</v>
       </c>
       <c r="B7" s="3" t="s">
@@ -4335,23 +4210,18 @@
         <v>333</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B9" s="10" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B10" s="10" t="s">
         <v>335</v>
       </c>
     </row>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
</xml_diff>